<commit_message>
feat(F-NAR-019): ATOM-AUT.ROU.001-04 Les fraises de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.ROU.001-04.xlsx
+++ b/stories/arbres/ATOM-AUT.ROU.001-04.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison puis rue du marché, le matin</t>
+          <t>chambre au rideau bleu, cuisine, rue du marché le matin</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut les fraises du marché tout de suite. Le cabas est vide. Une chose puis la suivante, elle goûte une fraise sucrée dans la rue.</t>
+          <t>La fenêtre respire, le rideau bleu gonfle. Sur l'anse du cabas rayé, un éclat de fraise — graine rose sèche — brille. Sarah veut les fraises du marché, maintenant. Elle saisit le cabas vide, pieds nus : l'anse glisse, le cabas tombe. Papa s'accroupit. Une chose, puis la suivante. À la porte, elle refuse de foncer. L'éclat penche vers le fond vide : la gourde manque. Elle la glisse. Au coin des barquettes, l'éclat porte une goutte de jus.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le rideau bleu se soulève avec le vent. Il gonfle comme une petite voile. Un anneau frotte la tringle, tout doux. Un carré de lumière glisse sur le plancher. Dehors, on pose déjà des caisses. Une charrette roule tout loin. Ça sent les fruits, même d'ici. Une caisse racle le pavé, tout loin. Sarah, tu vois le rideau ? Oui, papa. Il danse. Le marché commence, tout doucement. En ce moment, Sarah est encore au lit. Elle a envie des fraises, tout de suite. On y va maintenant ? Sarah prend le cabas rayé près de la porte. Le cabas est vide, tout plat. Elle n'a pas encore de chaussures. Les fraises seront là. D'abord notre matin. Une chose, puis la suivante. Sarah repose le cabas. Le tissu rayé tombe contre le mur. J'ai trop faim pour attendre. Alors on déjeune ici, d'abord. Après, tu auras encore faim pour les fraises. On se lève ? Oui. Sarah pousse le drap. Ses pieds trouvent le parquet lisse. Le parquet est un peu frais. Le t-shirt blanc, sur la commode.</t>
+          <t>La fenêtre respire, et le rideau bleu gonfle. Un anneau frotte la tringle, sec. Un carré de soleil glisse sur le plancher. Dehors, une charrette racle le pavé. L'odeur des fruits grimpe l'escalier. Près de la porte, le cabas rayé attend. Sur l'anse, un éclat de fraise brille. C'est une graine rose, sèche, coincée dans le tissage. Sarah la touche du doigt, puis la laisse. Sarah, tu entends la charrette ? Oui, papa. Ce sont les fraises ! Le marché s'installe, dans la rue. En ce moment, Sarah saute du lit. On y va, maintenant ! Elle attrape le cabas vide, d'un coup. Le tissu plat claque contre ses genoux. Ses pieds nus cherchent le parquet. Le bois est frais, lisse. Elle pousse vers la porte. L'anse glisse entre ses doigts. Le cabas tombe à plat. Il part ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Une chose, puis la suivante. Sarah repose le cabas. Le tissu rayé tombe contre le mur. J'ai trop faim pour attendre. Alors on déjeune ici, d'abord. On se lève ? Oui. Sarah pousse le drap. Ses orteils trouvent le parquet. Le t-shirt blanc, sur la commode.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le rideau bleu se soulève avec le vent. Il gonfle comme une petite voile. Un anneau frotte la tringle, tout doux. Un carré de lumière glisse sur le plancher. Dehors, on pose déjà des caisses. Une charrette roule tout loin. Ça sent les fruits, même d'ici. Une caisse racle le pavé, tout loin. Sarah, tu vois le rideau ? Oui, papa. Il danse. Le marché commence, tout doucement. En ce moment, Sarah est encore au lit. Elle a envie des fraises, tout de suite. On y va maintenant ? Sarah prend le cabas rayé près de la porte. Le cabas est vide, tout plat. Elle n'a pas encore de chaussures. Les fraises seront là. D'abord notre matin. Une chose, puis la suivante. Sarah repose le cabas. Le tissu rayé tombe contre le mur. J'ai trop faim pour attendre. Alors on déjeune ici, d'abord. Après, tu auras encore faim pour les fraises. On se lève ? Oui. Sarah pousse le drap. Ses pieds trouvent le parquet lisse. Le parquet est un peu frais. Le t-shirt blanc, sur la commode.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La fenêtre respire, et le rideau bleu gonfle. Un anneau frotte la tringle, sec. Un carré de soleil glisse sur le plancher. Dehors, une charrette racle le pavé. L'odeur des fruits grimpe l'escalier. Près de la porte, le cabas rayé attend. Sur l'anse, un &lt;emphasis level="moderate"&gt;éclat de fraise&lt;/emphasis&gt; brille. C'est une graine rose, sèche, coincée dans le tissage. Sarah la touche du doigt, puis la laisse. Sarah, tu entends la charrette ? Oui, papa. Ce sont les fraises ! Le marché s'installe, dans la rue. En ce moment, Sarah saute du lit. On y va, maintenant ! Elle attrape le cabas vide, d'un coup. Le tissu plat claque contre ses genoux. Ses pieds nus cherchent le parquet. Le bois est frais, lisse. Elle pousse vers la porte. L'anse glisse entre ses doigts. Le cabas tombe à plat. Il part ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Une chose, puis la suivante. Sarah repose le cabas. Le tissu rayé tombe contre le mur. J'ai trop faim pour attendre. Alors on déjeune ici, d'abord. On se lève ? Oui. Sarah pousse le drap. Ses orteils trouvent le parquet. Le t-shirt blanc, sur la commode.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil entre. Zoé ouvre les yeux. Papa dit : &lt;emphasis&gt;une&lt;/emphasis&gt; étape après l'autre. D'abord se lever. Puis s'habiller. Puis déjeuner. Puis le sac. Zoé se lève. C'est l'étape dite. Elle met le t-shirt. Une étape après l'autre. Elle s'assoit à table. Elle mange. Elle range le bol. Puis elle prend le sac. Papa dit : tu as fait une étape après l'autre. [pause]</t>
+          <t>La fenêtre respire, et le rideau bleu gonfle. Un anneau frotte la tringle, sec. Un carré de soleil glisse sur le plancher. Dehors, une charrette racle le pavé. L'odeur des fruits grimpe l'escalier. Près de la porte, le cabas rayé attend. Sur l'anse, un &lt;emphasis&gt;éclat de fraise&lt;/emphasis&gt; brille. C'est une graine rose, sèche, coincée dans le tissage. Sarah la touche du doigt, puis la laisse. Sarah, tu entends la charrette ? Oui, papa. Ce sont les fraises ! Le marché s'installe, dans la rue. En ce moment, Sarah saute du lit. On y va, maintenant ! Elle attrape le cabas vide, d'un coup. Le tissu plat claque contre ses genoux. Ses pieds nus cherchent le parquet. Le bois est frais, lisse. Elle pousse vers la porte. L'anse glisse entre ses doigts. Le cabas tombe à plat. Il part ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Une chose, puis la suivante. Sarah repose le cabas. Le tissu rayé tombe contre le mur. J'ai trop faim pour attendre. Alors on déjeune ici, d'abord. On se lève ? Oui. Sarah pousse le drap. Ses orteils trouvent le parquet. Le t-shirt blanc, sur la commode. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de fraise</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,46 +1321,53 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_les_fraises_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le rideau bleu se soulève avec le vent.
-narrateur|Il gonfle comme une petite voile.
-narrateur|Un anneau frotte la tringle, tout doux.
-narrateur|Un carré de lumière glisse sur le plancher.
-narrateur|Dehors, on pose déjà des caisses.
-narrateur|Une charrette roule tout loin.
-narrateur|Ça sent les fruits, même d'ici.
-narrateur|Une caisse racle le pavé, tout loin.
-papa|Sarah, tu vois le rideau ?
+          <t>narrateur|La fenêtre respire, et le rideau bleu gonfle.
+narrateur|Un anneau frotte la tringle, sec.
+narrateur|Un carré de soleil glisse sur le plancher.
+narrateur|Dehors, une charrette racle le pavé.
+narrateur|L'odeur des fruits grimpe l'escalier.
+narrateur|Près de la porte, le cabas rayé attend.
+narrateur|Sur l'anse, un éclat de fraise brille.
+narrateur|C'est une graine rose, sèche, coincée dans le tissage.
+narrateur|Sarah la touche du doigt, puis la laisse.
+papa|Sarah, tu entends la charrette ?
 enfant-f|Oui, papa.
-enfant-f|Il danse.
-maman|Le marché commence, tout doucement.
-narrateur|En ce moment, Sarah est encore au lit.
-narrateur|Elle a envie des fraises, tout de suite.
-enfant-f|On y va maintenant ?
-narrateur|Sarah prend le cabas rayé près de la porte.
-narrateur|Le cabas est vide, tout plat.
-narrateur|Elle n'a pas encore de chaussures.
-maman|Les fraises seront là.
-papa|D'abord notre matin.
+enfant-f|Ce sont les fraises !
+maman|Le marché s'installe, dans la rue.
+narrateur|En ce moment, Sarah saute du lit.
+enfant-f|On y va, maintenant !
+narrateur|Elle attrape le cabas vide, d'un coup.
+narrateur|Le tissu plat claque contre ses genoux.
+narrateur|Ses pieds nus cherchent le parquet.
+narrateur|Le bois est frais, lisse.
+narrateur|Elle pousse vers la porte.
+narrateur|L'anse glisse entre ses doigts.
+narrateur|Le cabas tombe à plat.
+enfant-f|Il part !
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
 papa|Une chose, puis la suivante.
 narrateur|Sarah repose le cabas.
 narrateur|Le tissu rayé tombe contre le mur.
 enfant-f|J'ai trop faim pour attendre.
 maman|Alors on déjeune ici, d'abord.
-maman|Après, tu auras encore faim pour les fraises.
 papa|On se lève ?
 enfant-f|Oui.
 narrateur|Sarah pousse le drap.
-narrateur|Ses pieds trouvent le parquet lisse.
-narrateur|Le parquet est un peu frais.
+narrateur|Ses orteils trouvent le parquet.
 maman|Le t-shirt blanc, sur la commode.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>rideau</t>
+          <t>rideau,charrette</t>
         </is>
       </c>
     </row>
@@ -1392,12 +1399,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah veut les fraises. Comment se prépare-t-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah veut les &lt;emphasis level="moderate"&gt;fraises&lt;/emphasis&gt;. Comment se prépare-t-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Zoé se prépare. Que fait-elle ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah veut les &lt;emphasis&gt;fraises&lt;/emphasis&gt;. Comment se prépare-t-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1460,7 +1467,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1468,10 +1475,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1486,34 +1493,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>fraises</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1522,23 +1533,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=une_chose_puis_la_suivante; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1571,17 +1582,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah enfile le t-shirt. Le coton est encore un peu tiède. Je suis habillée. La cuisine, maintenant. La nappe à carreaux est déjà mise. Ça sent le yaourt et le miel. Tu veux un peu de miel ? Oui, un peu. Sarah s'assoit. Elle pose les pieds par terre. Le miel est sucré sur la cuillère. Tu as encore faim pour le marché ? Un peu, oui. C'est bien. Les fraises aiment ça. Merci, Sarah. Ensuite, le cabas.</t>
+          <t>Papa s'accroupit à la même hauteur. Le t-shirt, d'abord. Sarah prend le coton sur la commode. Le t-shirt est tiède, un peu froissé. Elle l'enfile sans se presser. Je suis habillée. La cuisine, maintenant. Sarah marche vers la table. La nappe à carreaux sent le pain. Deux bols blancs attendent. Tu veux du yaourt ? Oui, un peu. Sarah s'assoit. Elle pose les pieds par terre. Le yaourt est froid sur la cuillère. Tu as faim pour le marché ? Un peu, oui. Alors les fraises, après. Dehors, une caisse racle le pavé. Je les entends. Ensuite, le cabas. Le cabas rayé attend près du mur. Sarah le soulève. Le tissu tombe droit.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah enfile le t-shirt. Le coton est encore un peu tiède. Je suis habillée. La cuisine, maintenant. La nappe à carreaux est déjà mise. Ça sent le yaourt et le miel. Tu veux un peu de miel ? Oui, un peu. Sarah s'assoit. Elle pose les pieds par terre. Le miel est sucré sur la cuillère. Tu as encore faim pour le marché ? Un peu, oui. C'est bien. Les fraises aiment ça. Merci, Sarah. Ensuite, le cabas.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa s'accroupit à la même hauteur. Le t-shirt, d'abord. Sarah prend le coton sur la commode. Le t-shirt est tiède, un peu froissé. Elle l'enfile sans se presser. Je suis habillée. La cuisine, maintenant. Sarah marche vers la table. La nappe à carreaux sent le pain. Deux bols blancs attendent. Tu veux du yaourt ? Oui, un peu. Sarah s'assoit. Elle pose les pieds par terre. Le yaourt est froid sur la cuillère. Tu as faim pour le marché ? Un peu, oui. Alors les fraises, après. Dehors, une caisse racle le pavé. Je les entends. Ensuite, le &lt;emphasis level="moderate"&gt;cabas&lt;/emphasis&gt;. Le cabas rayé attend près du mur. Sarah le soulève. Le tissu tombe droit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Zoé a fait &lt;emphasis&gt;une&lt;/emphasis&gt; étape après l'autre. Lever, habiller, déjeuner, sac. [pause]</t>
+          <t>Papa s'accroupit à la même hauteur. Le t-shirt, d'abord. Sarah prend le coton sur la commode. Le t-shirt est tiède, un peu froissé. Elle l'enfile sans se presser. Je suis habillée. La cuisine, maintenant. Sarah marche vers la table. La nappe à carreaux sent le pain. Deux bols blancs attendent. Tu veux du yaourt ? Oui, un peu. Sarah s'assoit. Elle pose les pieds par terre. Le yaourt est froid sur la cuillère. Tu as faim pour le marché ? Un peu, oui. Alors les fraises, après. Dehors, une caisse racle le pavé. Je les entends. Ensuite, le &lt;emphasis&gt;cabas&lt;/emphasis&gt;. Le cabas rayé attend près du mur. Sarah le soulève. Le tissu tombe droit. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1628,7 +1639,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1636,10 +1647,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1662,11 +1673,11 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>cabas</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
         <v>450</v>
@@ -1676,16 +1687,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1694,10 +1705,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1710,28 +1721,40 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=t_shirt_puis_table_puis_cabas; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah enfile le t-shirt.
-narrateur|Le coton est encore un peu tiède.
+          <t>narrateur|Papa s'accroupit à la même hauteur.
+papa|Le t-shirt, d'abord.
+narrateur|Sarah prend le coton sur la commode.
+narrateur|Le t-shirt est tiède, un peu froissé.
+narrateur|Elle l'enfile sans se presser.
 enfant-f|Je suis habillée.
-papa|La cuisine, maintenant.
-narrateur|La nappe à carreaux est déjà mise.
-narrateur|Ça sent le yaourt et le miel.
-maman|Tu veux un peu de miel ?
+maman|La cuisine, maintenant.
+narrateur|Sarah marche vers la table.
+narrateur|La nappe à carreaux sent le pain.
+narrateur|Deux bols blancs attendent.
+maman|Tu veux du yaourt ?
 enfant-f|Oui, un peu.
 narrateur|Sarah s'assoit.
 narrateur|Elle pose les pieds par terre.
-narrateur|Le miel est sucré sur la cuillère.
-papa|Tu as encore faim pour le marché ?
+narrateur|Le yaourt est froid sur la cuillère.
+papa|Tu as faim pour le marché ?
 enfant-f|Un peu, oui.
-maman|C'est bien.
-maman|Les fraises aiment ça.
-papa|Merci, Sarah.
-maman|Ensuite, le cabas.</t>
+maman|Alors les fraises, après.
+narrateur|Dehors, une caisse racle le pavé.
+enfant-f|Je les entends.
+papa|Ensuite, le cabas.
+narrateur|Le cabas rayé attend près du mur.
+narrateur|Sarah le soulève.
+narrateur|Le tissu tombe droit.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tissu,bol</t>
         </is>
       </c>
     </row>
@@ -1758,17 +1781,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend le cabas rayé. Le cabas sent encore le linge. La gourde est fraîche, tout au fond. Les fraises sont tout près ? Oui, maman. Sarah met ses chaussures. On prend le cabas ? Oui, papa. Papa ouvre la porte. Sarah donne la main. La rue sent les fruits. Un panier passe, tout plein. Les fraises ! Choisis. Sarah choisit une barquette rouge. Une fraise est déjà un peu chaude. Tu la goûtes ? Elle est sucrée. Un peu de jus rouge reste sur le doigt. Tu l'as choisie, celle-là. Une caisse racle encore, tout près. On en prend une autre ? Celle-ci, la plus rouge.</t>
+          <t>Sarah met ses chaussures. On prend le cabas ? Oui, papa. Papa ouvre la porte. Un souffle pousse le rideau bleu. Le cabas se balance, vide au fond. Les fraises ! Sarah veut courir, l'anse à la main. Elle veut descendre, sans regarder. Sarah refuse de foncer. Attends, je regarde. Sur l'anse, l'éclat de fraise tremble. La graine penche vers le fond du cabas. Il manque la gourde ! Elle est où, la gourde ? Dans la cuisine, au frais. Sarah revient vers la table. Elle glisse la gourde froide au fond. L'éclat de fraise tient, coincé. Merci, Sarah. On y va ? Oui, le cabas est prêt. Sarah donne la main. La rue sent les fruits. Un panier passe, plein. Les voilà ! Au coin des barquettes. Sarah choisit une barquette rouge. Une fraise est chaude sous le soleil. Tu la goûtes ? Elle est sucrée. Un peu de jus rouge reste sur le doigt.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend le cabas rayé. Le cabas sent encore le linge. La gourde est fraîche, tout au fond. Les fraises sont tout près ? Oui, maman. Sarah met ses chaussures. On prend le cabas ? Oui, papa. Papa ouvre la porte. Sarah donne la main. La rue sent les fruits. Un panier passe, tout plein. Les fraises ! Choisis. Sarah choisit une barquette rouge. Une fraise est déjà un peu chaude. Tu la goûtes ? Elle est sucrée. Un peu de jus rouge reste sur le doigt. Tu l'as choisie, celle-là. Une caisse racle encore, tout près. On en prend une autre ? Celle-ci, la plus rouge.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah met ses chaussures. On prend le cabas ? Oui, papa. Papa ouvre la porte. Un souffle pousse le rideau bleu. Le cabas se balance, vide au fond. Les fraises ! Sarah veut courir, l'anse à la main. Elle veut descendre, sans regarder. Sarah refuse de foncer. Attends, je regarde. Sur l'anse, l'&lt;emphasis level="moderate"&gt;éclat de fraise&lt;/emphasis&gt; tremble. La graine penche vers le fond du cabas. Il manque la gourde ! Elle est où, la gourde ? Dans la cuisine, au frais. Sarah revient vers la table. Elle glisse la gourde froide au fond. L'éclat de fraise tient, coincé. Merci, Sarah. On y va ? Oui, le cabas est prêt. Sarah donne la main. La rue sent les fruits. Un panier passe, plein. Les voilà ! Au coin des barquettes. Sarah choisit une barquette rouge. Une fraise est chaude sous le soleil. Tu la goûtes ? Elle est sucrée. Un peu de jus rouge reste sur le doigt.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa ouvre la porte. Zoé donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Sarah met ses chaussures. On prend le cabas ? Oui, papa. Papa ouvre la porte. Un souffle pousse le rideau bleu. Le cabas se balance, vide au fond. Les fraises ! Sarah veut courir, l'anse à la main. Elle veut descendre, sans regarder. Sarah refuse de foncer. Attends, je regarde. Sur l'anse, l'&lt;emphasis&gt;éclat de fraise&lt;/emphasis&gt; tremble. La graine penche vers le fond du cabas. Il manque la gourde ! Elle est où, la gourde ? Dans la cuisine, au frais. Sarah revient vers la table. Elle glisse la gourde froide au fond. L'éclat de fraise tient, coincé. Merci, Sarah. On y va ? Oui, le cabas est prêt. Sarah donne la main. La rue sent les fruits. Un panier passe, plein. Les voilà ! Au coin des barquettes. Sarah choisit une barquette rouge. Une fraise est chaude sous le soleil. Tu la goûtes ? Elle est sucrée. Un peu de jus rouge reste sur le doigt. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1815,7 +1838,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1823,10 +1846,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1849,30 +1872,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de fraise</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1881,10 +1904,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1895,37 +1918,50 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_l_éclat_montre_la_gourde; tempo=naturel; sourire=franc; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah prend le cabas rayé.
-narrateur|Le cabas sent encore le linge.
-narrateur|La gourde est fraîche, tout au fond.
-maman|Les fraises sont tout près ?
-enfant-f|Oui, maman.
-narrateur|Sarah met ses chaussures.
+          <t>narrateur|Sarah met ses chaussures.
 papa|On prend le cabas ?
 enfant-f|Oui, papa.
 narrateur|Papa ouvre la porte.
+narrateur|Un souffle pousse le rideau bleu.
+narrateur|Le cabas se balance, vide au fond.
+enfant-f|Les fraises !
+narrateur|Sarah veut courir, l'anse à la main.
+narrateur|Elle veut descendre, sans regarder.
+narrateur|Sarah refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Sur l'anse, l'éclat de fraise tremble.
+narrateur|La graine penche vers le fond du cabas.
+enfant-f|Il manque la gourde !
+maman|Elle est où, la gourde ?
+enfant-f|Dans la cuisine, au frais.
+narrateur|Sarah revient vers la table.
+narrateur|Elle glisse la gourde froide au fond.
+narrateur|L'éclat de fraise tient, coincé.
+papa|Merci, Sarah.
+papa|On y va ?
+enfant-f|Oui, le cabas est prêt.
 narrateur|Sarah donne la main.
 narrateur|La rue sent les fruits.
-narrateur|Un panier passe, tout plein.
-enfant-f|Les fraises !
-maman|Choisis.
+narrateur|Un panier passe, plein.
+enfant-f|Les voilà !
+maman|Au coin des barquettes.
 narrateur|Sarah choisit une barquette rouge.
-narrateur|Une fraise est déjà un peu chaude.
+narrateur|Une fraise est chaude sous le soleil.
 papa|Tu la goûtes ?
 enfant-f|Elle est sucrée.
-narrateur|Un peu de jus rouge reste sur le doigt.
-maman|Tu l'as choisie, celle-là.
-narrateur|Une caisse racle encore, tout près.
-papa|On en prend une autre ?
-enfant-f|Celle-ci, la plus rouge.</t>
+narrateur|Un peu de jus rouge reste sur le doigt.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte</t>
+          <t>porte,rue</t>
         </is>
       </c>
     </row>
@@ -1952,17 +1988,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai du rouge sur le doigt. C'est le marché. Une chose, puis la suivante, et les fraises étaient là. Le rideau, derrière eux, danse encore. Bravo, Sarah. Le jus sucré reste chaud sur son doigt.</t>
+          <t>J'ai du rouge sur le doigt. C'est le marché. Sur l'anse, l'éclat de fraise porte une goutte. La graine rose est collante, un peu chaude. Elle a voyagé. Comme toi. Le rideau bleu danse à la fenêtre. Le jus sucré reste chaud sur son doigt.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai du rouge sur le doigt. C'est le marché. Une chose, puis la suivante, et les fraises étaient là. Le rideau, derrière eux, danse encore. Bravo, Sarah. Le jus sucré reste chaud sur son doigt.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;J'ai du rouge sur le doigt. C'est le marché. Sur l'anse, l'&lt;emphasis level="moderate"&gt;éclat de fraise&lt;/emphasis&gt; porte une goutte. La graine rose est collante, un peu chaude. Elle a voyagé. Comme toi. Le rideau bleu danse à la fenêtre. Le jus sucré reste chaud sur son doigt.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;J'ai du rouge sur le doigt. C'est le marché. Sur l'anse, l'&lt;emphasis&gt;éclat de fraise&lt;/emphasis&gt; porte une goutte. La graine rose est collante, un peu chaude. Elle a voyagé. Comme toi. Le rideau bleu danse à la fenêtre. Le jus sucré reste chaud sur son doigt.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2009,18 +2045,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2029,12 +2065,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2043,17 +2079,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de fraise</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2062,11 +2102,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2075,29 +2115,40 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_éclat_porte_une_goutte_de_jus; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>enfant-f|J'ai du rouge sur le doigt.
 maman|C'est le marché.
-papa|Une chose, puis la suivante, et les fraises étaient là.
-narrateur|Le rideau, derrière eux, danse encore.
-maman|Bravo, Sarah.
+narrateur|Sur l'anse, l'éclat de fraise porte une goutte.
+narrateur|La graine rose est collante, un peu chaude.
+enfant-f|Elle a voyagé.
+papa|Comme toi.
+narrateur|Le rideau bleu danse à la fenêtre.
 narrateur|Le jus sucré reste chaud sur son doigt.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>fruits</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2217,6 +2268,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>